<commit_message>
Stage 8 review fixes: E-006
</commit_message>
<xml_diff>
--- a/output/archive/WestravelleData/Stability/OD18/WA-2019-010/Results/Approved/OD18_PULLS_AND_SUITABILITY_RESULTS_Rev03.xlsx
+++ b/output/archive/WestravelleData/Stability/OD18/WA-2019-010/Results/Approved/OD18_PULLS_AND_SUITABILITY_RESULTS_Rev03.xlsx
@@ -171,9 +171,9 @@
     <author>Andrea Tucker</author>
   </authors>
   <commentList>
-    <comment ref="D3" authorId="0" shapeId="0">
+    <comment ref="B3" authorId="0" shapeId="0">
       <text>
-        <t>Recommendation accepted for the next pack configuration.</t>
+        <t>Carry the desiccant recommendation into the next pack protocol.</t>
       </text>
     </comment>
   </commentList>
@@ -611,7 +611,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Six-month stability of OD-18 powder under humidity challenge at 25 °C/60% RH and 40 °C/75% RH. Pulls at 0, 3 and 6 months; the three-month interim review was completed on 13 May 2019.</t>
+          <t>Six-month stability of OD-18 powder under humidity challenge at 25 °C/60% RH, 30 °C/65% RH and 40 °C/75% RH. Initial analysis followed by pulls at 1, 3 and 6 months; the three-month interim review was completed on 13 May 2019.</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Assay at time zero was 100.2 % label claim. The assay drift seen at the warm condition followed moisture uptake, not chemical instability. Odraverne specified desiccant protection for the next pack configuration.</t>
+          <t>Assay at time zero was 100.2 % label claim. The project review attributed assay drift to moisture uptake. Water results fluctuate and impurities also increase at the warm condition; this table alone does not exclude chemical degradation. Odraverne specified desiccant protection for the next pack configuration.</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Stability results and total impurities chart</t>
+          <t>Stability results and assay chart</t>
         </is>
       </c>
     </row>
@@ -712,7 +712,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Assay as % label claim (HPLC). Impurities as % area. Water by Karl Fischer. Pulls from the ICH chamber programme as recorded on the batch card.</t>
+          <t>Assay as % label claim (HPLC). Impurities as % area. Water by Karl Fischer. Pulls from the ICH chamber programme as recorded on the batch card. Time zero is one initial analysis shared by all storage conditions; repeated initial rows do not represent separate pulls.</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1163,91 +1163,70 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Humidity challenge: configurations and storage</t>
+          <t>Humidity challenge: storage and interpretation</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Powder held in open dish and in the two sealed configurations below, at both conditions. Sealed samples were opened only at the pull.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Condition</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>25 °C/60% RH</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Long-term reference</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Configuration</t>
+          <t>30 °C/65% RH</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Storage</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Notes</t>
+          <t>Intermediate</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Open dish</t>
+          <t>40 °C/75% RH</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>25 °C/60% RH and 40 °C/75% RH</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Worst-case exposure, reference only</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Sealed bottle, no desiccant</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>25 °C/60% RH and 40 °C/75% RH</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Current pack configuration</t>
-        </is>
-      </c>
-    </row>
+          <t>Accelerated</t>
+        </is>
+      </c>
+    </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Sealed bottle with desiccant canister</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>25 °C/60% RH and 40 °C/75% RH</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Proposed for the next pack configuration</t>
-        </is>
-      </c>
-    </row>
-    <row r="8"/>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Chamber logs were reviewed at each pull. No alarm affected the warm condition during the study.</t>
+          <t>Pack configurations and chamber history are recorded on the batch card and chamber logs. The result table does not separate sealed and unsealed presentations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Desiccant protection was specified for the next pack configuration; effectiveness of that future configuration is not established by these results.</t>
         </is>
       </c>
     </row>
@@ -1263,7 +1242,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1275,27 +1254,17 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Agreed actions</t>
+          <t>Packaging disposition and follow-up</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Action</t>
+          <t>Item</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Due</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -1304,66 +1273,36 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Specify desiccant canister in the next pack configuration</t>
+          <t>Desiccant protection for the next pack configuration</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Dr L. Wu</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>30 Sep 2019</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Agreed with Odraverne</t>
+          <t>Specified by Odraverne</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Add moisture-uptake check at the three-month pull for future humidity programmes</t>
+          <t>Future pack assessment</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Dr A. Penrose</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>31 Dec 2019</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Any confirmatory protocol, dates and owners are to be agreed separately.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Re-run assay on retained samples from the six-month pull after the moisture check</t>
+          <t>Repeat analysis / deviation history</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>S. Mahmood</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>15 Sep 2019</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Closed</t>
+          <t>Refer to the approved sequence sheets; no additional repeat results are reported here.</t>
         </is>
       </c>
     </row>

</xml_diff>